<commit_message>
Updated OCR website UI and camera
</commit_message>
<xml_diff>
--- a/scanned_cards.xlsx
+++ b/scanned_cards.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bbc5a9cab421d4b2/Desktop/business-card-ocr/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="11_2B59D2BFD3A0DD679D62D4F0509818B242BDE3D0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AB6EBA50-0832-468C-AA32-13AD19B9C628}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{A329D440-8F6B-4957-8D79-93001E75AB99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="47">
   <si>
     <t>OCR Text</t>
   </si>
@@ -144,6 +144,33 @@
   </si>
   <si>
     <t>&gt; b -aroteal Swestik industrial Complex, Ni Times Ot India Sector Ld 40, Gala 0.10, Plot No 23 PCNTDA Bhosan Pune 4: "eo . ages, Cillthel, Pune 41106)</t>
+  </si>
+  <si>
+    <t>INVICTUS S™</t>
+  </si>
+  <si>
+    <t>EMPOWERING INDUSTRIES WITH</t>
+  </si>
+  <si>
+    <t>© Regd. Add.: Sr. No. 66/1, Near HDFC Bank, |, New Sangvi, Pune - 411 061.</t>
+  </si>
+  <si>
+    <t>EE EE</t>
+  </si>
+  <si>
+    <t>EMPOWERING INDUSTRIES WITH.</t>
+  </si>
+  <si>
+    <t>nvictusmachinesolution.com</t>
+  </si>
+  <si>
+    <t>© Regd. Add.: Sr No. 66/1, Near HDFC Bank, ¢, New Sanevi, Pune - 411 061.</t>
+  </si>
+  <si>
+    <t>EMPOWERING INDUSTRIES WITH |</t>
+  </si>
+  <si>
+    <t>(© Regd. Add.: Sr. No. 66/1, Near HDFC Bank, ¢, New Sangvi, Pune - 411 061.</t>
   </si>
 </sst>
 </file>
@@ -483,16 +510,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="2" max="2" width="22.77734375" customWidth="1"/>
-    <col min="3" max="3" width="28.88671875" customWidth="1"/>
-    <col min="4" max="4" width="21.21875" customWidth="1"/>
-    <col min="5" max="5" width="39.77734375" customWidth="1"/>
-    <col min="6" max="6" width="52.44140625" customWidth="1"/>
-    <col min="10" max="10" width="17.5546875" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
@@ -646,6 +665,72 @@
         <v>20</v>
       </c>
     </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="C11" t="s">
+        <v>15</v>
+      </c>
+      <c r="E11" t="s">
+        <v>38</v>
+      </c>
+      <c r="G11" t="s">
+        <v>39</v>
+      </c>
+      <c r="H11" t="s">
+        <v>17</v>
+      </c>
+      <c r="I11" t="s">
+        <v>40</v>
+      </c>
+      <c r="J11" t="s">
+        <v>19</v>
+      </c>
+      <c r="K11" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="E12" t="s">
+        <v>41</v>
+      </c>
+      <c r="G12" t="s">
+        <v>42</v>
+      </c>
+      <c r="H12" t="s">
+        <v>43</v>
+      </c>
+      <c r="I12" t="s">
+        <v>44</v>
+      </c>
+      <c r="J12" t="s">
+        <v>19</v>
+      </c>
+      <c r="K12" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="C13" t="s">
+        <v>15</v>
+      </c>
+      <c r="E13" t="s">
+        <v>41</v>
+      </c>
+      <c r="G13" t="s">
+        <v>45</v>
+      </c>
+      <c r="H13" t="s">
+        <v>17</v>
+      </c>
+      <c r="I13" t="s">
+        <v>46</v>
+      </c>
+      <c r="J13" t="s">
+        <v>19</v>
+      </c>
+      <c r="K13" t="s">
+        <v>20</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>